<commit_message>
Append ten independently source-reviewed NJU academic profiles with live conservation checks
</commit_message>
<xml_diff>
--- a/site/exports/nju-social-sciences.xlsx
+++ b/site/exports/nju-social-sciences.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -622,11 +622,65 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>社会学院/社会学系</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>No personal degree-stage advisor identified in accepted sources.；Award years/dates left null; educational range endpoints are not automatically award dates.；Directory 全职教师 label and 2024 CV do not independently prove present employment.；PDF text read, no original PDF retained and screenshot failed cache miss.；目录原生pagem.htm与实际读取page3.htm共享文章ID；不声称未读模板字节等价。；校区、院校985与地域分类未独立规范化。；本批选取部分职业事实，不是全履历或现职认证。</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；部分公开职业资料；非完整履历或当前人事在岗证明；公开教学事实（非本人求学学历；教学／课程开设时间不是入学、授位或任职起点；不计入教育、任职、论文、导师统计及师承图）：城市社会学；未披露；教学／课程开设时间：时间未披露；来源授课栏目；具体授课角色与本期开课未知。；来源ID：nju-huxiaowu-profile；https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm | 城市生活方式；未披露；教学／课程开设时间：时间未披露；来源授课栏目；具体授课角色与本期开课未知。；来源ID：nju-huxiaowu-profile；https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm | 贫困与发展；未披露；教学／课程开设时间：时间未披露；来源授课栏目；具体授课角色与本期开课未知。；来源ID：nju-huxiaowu-profile；https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm | 社会营销；未披露；教学／课程开设时间：时间未披露；来源授课栏目；具体授课角色与本期开课未知。；来源ID：nju-huxiaowu-profile；https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:K4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -638,7 +692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1192,8 +1246,327 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>南昌大学</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Study interval end is not asserted to be degree-award date. Legal awarding entity and formal dissertation advisor remain unresolved. Award support is the explicit qualification 学士学位/硕士学位, not graduation alone; department retained separately, no degree-discipline invented.</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>本批未独立规范化院校985及地域分类，保留unknown。</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/_upload/article/files/41/95/7809386148a4a4f31250cdd315c6/830e66b4-234e-41f3-b1e2-ebf2578e2911.pdf</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Study interval end is not asserted to be degree-award date. Legal awarding entity and formal dissertation advisor remain unresolved. Award support is the explicit qualification 学士学位/硕士学位, not graduation alone; department retained separately, no degree-discipline invented.</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>本批未独立规范化院校985及地域分类，保留unknown。</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/_upload/article/files/41/95/7809386148a4a4f31250cdd315c6/830e66b4-234e-41f3-b1e2-ebf2578e2911.pdf</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>社会学</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Study interval end is not asserted to be degree-award date. Legal awarding entity and formal dissertation advisor remain unresolved.</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>本批未独立规范化院校985及地域分类，保留unknown。</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/_upload/article/files/41/95/7809386148a4a4f31250cdd315c6/830e66b4-234e-41f3-b1e2-ebf2578e2911.pdf</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>自2007年始任教 supports teaching start only; does not date associate-professor appointment.</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/_upload/article/files/41/95/7809386148a4a4f31250cdd315c6/830e66b4-234e-41f3-b1e2-ebf2578e2911.pdf</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>副教授</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S8"/>
+  <autoFilter ref="A1:S13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -1202,6 +1575,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1304,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1495,8 +1873,120 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>传承与升华——城市旅游开发与营销战略</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>专著；book</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>官网及简历书目；未核出版社元数据或全文。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>作者由简历个人专著栏目支持；原PDF未留存，未作视觉核验。</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>城市张力——咖啡馆与生活方式转型</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>专著；book</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>官网及简历书目；未核出版社元数据或全文。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>作者由简历个人专著栏目支持；原PDF未留存，未作视觉核验。</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L3"/>
+  <autoFilter ref="A1:L5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -1504,6 +1994,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1515,13 +2011,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="36.4" customWidth="1" min="2" max="2"/>
+    <col width="39.2" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="53.2" customWidth="1" min="4" max="4"/>
+    <col width="58.8" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -1712,13 +2208,165 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>nju-huxiaowu-cv</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/_upload/article/files/41/95/7809386148a4a4f31250cdd315c6/830e66b4-234e-41f3-b1e2-ebf2578e2911.pdf</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>official_cv_pdf_text_extraction</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>nju-huxiaowu-profile</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/9a/6a/c58987a694890/page3.htm</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>official_profile_body</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>nju-sociology-roster</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/qzjs/listm.htm</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>official_roster_body</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>胡小武</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>nju-sociology-roster-browser</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>https://sociology.nju.edu.cn/qzjs/listm.htm</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>parent_actual_cloud_browser_directory_href</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>nju</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>南京大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:G9"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>